<commit_message>
Fig. 3d and ED Fig. 7 on the literature Ru parameters; Source Data, READMEs, text-number table
Fig. 3d: benchmark-bed Ru/C + recovery at r = 0.90-0.97; own bed as squares at 8 wt% Ru, 490 kg m-3 with bars over
5-10 wt% and 430-550 kg m-3, main and KAAP loops. ED Fig. 7 panel d bins the A_bed Ru content (5-10 wt%). Only the
files whose pixels or cell values changed are kept. fig2_ru_alpha_sweep.csv is parameter-independent and kept at its
committed version (cloud rerun differs by 1.6e-14 relative).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/source_data/SourceData_EDFig7.xlsx
+++ b/source_data/SourceData_EDFig7.xlsx
@@ -533,7 +533,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>analysis/nh3_mc_ru_actual_2026_10_06/draws.csv (Ru wins: Ru_A_bed &lt; Fe, or Ru_A &lt; Fe); bins of the drawn Ru content</t>
+          <t>analysis/nh3_mc_ru_actual_2026_10_06/draws.csv (Ru wins: Ru_A_bed &lt; Fe, or Ru_A &lt; Fe); 5 bins of the drawn A_bed Ru content (A_bed_wt_pct)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -642,7 +642,7 @@
         <v>5000</v>
       </c>
       <c r="E4" t="n">
-        <v>7.110423493907948</v>
+        <v>7.110423493907959</v>
       </c>
     </row>
     <row r="5">
@@ -657,19 +657,19 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.4798</v>
+        <v>0.3556</v>
       </c>
       <c r="D5" t="n">
         <v>5000</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.01433004794961779</v>
+        <v>-0.0942516738250303</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>A_bed: u and r, supported bed</t>
+          <t>A_bed: u and r, commercial Ru/C bed</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -678,19 +678,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.7998</v>
+        <v>0.6898</v>
       </c>
       <c r="D6" t="n">
         <v>5000</v>
       </c>
       <c r="E6" t="n">
-        <v>0.3687787202002459</v>
+        <v>0.1786261991028901</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>B: measured Ru catalysts, 90-94 % recovery</t>
+          <t>B: measured Ru catalysts, 90-97 % recovery</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -699,13 +699,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.9429999999999999</v>
+        <v>0.9466</v>
       </c>
       <c r="D7" t="n">
         <v>5000</v>
       </c>
       <c r="E7" t="n">
-        <v>4.35034782150187</v>
+        <v>4.926524813946543</v>
       </c>
     </row>
     <row r="8">
@@ -720,13 +720,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.9893999999999999</v>
+        <v>0.99</v>
       </c>
       <c r="D8" t="n">
         <v>5000</v>
       </c>
       <c r="E8" t="n">
-        <v>7.40586957209078</v>
+        <v>7.774046410924601</v>
       </c>
     </row>
   </sheetData>
@@ -826,10 +826,10 @@
         <v>594</v>
       </c>
       <c r="D4" t="n">
-        <v>0.003367003367003367</v>
+        <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.1902356902356902</v>
+        <v>0.3434343434343434</v>
       </c>
     </row>
     <row r="5">
@@ -843,10 +843,10 @@
         <v>662</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01208459214501511</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>0.2522658610271903</v>
+        <v>0.4078549848942598</v>
       </c>
     </row>
     <row r="6">
@@ -860,10 +860,10 @@
         <v>626</v>
       </c>
       <c r="D6" t="n">
-        <v>0.02715654952076677</v>
+        <v>0.01277955271565495</v>
       </c>
       <c r="E6" t="n">
-        <v>0.3146964856230032</v>
+        <v>0.476038338658147</v>
       </c>
     </row>
     <row r="7">
@@ -877,10 +877,10 @@
         <v>638</v>
       </c>
       <c r="D7" t="n">
-        <v>0.09090909090909091</v>
+        <v>0.08150470219435736</v>
       </c>
       <c r="E7" t="n">
-        <v>0.493730407523511</v>
+        <v>0.658307210031348</v>
       </c>
     </row>
     <row r="8">
@@ -894,10 +894,10 @@
         <v>572</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1975524475524476</v>
+        <v>0.243006993006993</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5646853146853147</v>
+        <v>0.6940559440559441</v>
       </c>
     </row>
     <row r="9">
@@ -911,10 +911,10 @@
         <v>634</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2586750788643533</v>
+        <v>0.4858044164037855</v>
       </c>
       <c r="E9" t="n">
-        <v>0.667192429022082</v>
+        <v>0.7649842271293376</v>
       </c>
     </row>
     <row r="10">
@@ -928,10 +928,10 @@
         <v>640</v>
       </c>
       <c r="D10" t="n">
-        <v>0.425</v>
+        <v>0.7515625</v>
       </c>
       <c r="E10" t="n">
-        <v>0.796875</v>
+        <v>0.875</v>
       </c>
     </row>
     <row r="11">
@@ -945,10 +945,10 @@
         <v>634</v>
       </c>
       <c r="D11" t="n">
-        <v>0.5788643533123028</v>
+        <v>0.88801261829653</v>
       </c>
       <c r="E11" t="n">
-        <v>0.8722397476340694</v>
+        <v>0.9274447949526814</v>
       </c>
     </row>
   </sheetData>
@@ -1042,135 +1042,135 @@
         <v>0.9</v>
       </c>
       <c r="B4" t="n">
-        <v>0.905</v>
+        <v>0.9087500000000001</v>
       </c>
       <c r="C4" t="n">
         <v>585</v>
       </c>
       <c r="D4" t="n">
-        <v>0.1709401709401709</v>
+        <v>0.2085470085470086</v>
       </c>
       <c r="E4" t="n">
-        <v>0.4205128205128205</v>
+        <v>0.4341880341880342</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>0.905</v>
+        <v>0.9087500000000001</v>
       </c>
       <c r="B5" t="n">
-        <v>0.91</v>
+        <v>0.9175</v>
       </c>
       <c r="C5" t="n">
         <v>603</v>
       </c>
       <c r="D5" t="n">
-        <v>0.1575456053067993</v>
+        <v>0.2321724709784411</v>
       </c>
       <c r="E5" t="n">
-        <v>0.4112769485903814</v>
+        <v>0.4461028192371476</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>0.91</v>
+        <v>0.9175</v>
       </c>
       <c r="B6" t="n">
-        <v>0.915</v>
+        <v>0.92625</v>
       </c>
       <c r="C6" t="n">
         <v>634</v>
       </c>
       <c r="D6" t="n">
-        <v>0.165615141955836</v>
+        <v>0.2602523659305994</v>
       </c>
       <c r="E6" t="n">
-        <v>0.4747634069400631</v>
+        <v>0.5488958990536278</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>0.915</v>
+        <v>0.92625</v>
       </c>
       <c r="B7" t="n">
-        <v>0.9199999999999999</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="C7" t="n">
         <v>634</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2050473186119874</v>
+        <v>0.2854889589905363</v>
       </c>
       <c r="E7" t="n">
-        <v>0.5078864353312302</v>
+        <v>0.5993690851735016</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>0.9199999999999999</v>
+        <v>0.9350000000000001</v>
       </c>
       <c r="B8" t="n">
-        <v>0.9249999999999999</v>
+        <v>0.94375</v>
       </c>
       <c r="C8" t="n">
         <v>638</v>
       </c>
       <c r="D8" t="n">
-        <v>0.2053291536050157</v>
+        <v>0.3072100313479624</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5078369905956113</v>
+        <v>0.6473354231974922</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>0.9249999999999999</v>
+        <v>0.94375</v>
       </c>
       <c r="B9" t="n">
-        <v>0.9299999999999999</v>
+        <v>0.9525</v>
       </c>
       <c r="C9" t="n">
         <v>649</v>
       </c>
       <c r="D9" t="n">
-        <v>0.2003081664098613</v>
+        <v>0.3235747303543914</v>
       </c>
       <c r="E9" t="n">
-        <v>0.5562403697996918</v>
+        <v>0.7503852080123267</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>0.9299999999999999</v>
+        <v>0.9525</v>
       </c>
       <c r="B10" t="n">
-        <v>0.9349999999999999</v>
+        <v>0.9612499999999999</v>
       </c>
       <c r="C10" t="n">
         <v>640</v>
       </c>
       <c r="D10" t="n">
-        <v>0.2546875</v>
+        <v>0.4171875</v>
       </c>
       <c r="E10" t="n">
-        <v>0.6234375</v>
+        <v>0.8296875</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0.9349999999999999</v>
+        <v>0.9612499999999999</v>
       </c>
       <c r="B11" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.97</v>
       </c>
       <c r="C11" t="n">
         <v>617</v>
       </c>
       <c r="D11" t="n">
-        <v>0.2382495948136143</v>
+        <v>0.4376012965964344</v>
       </c>
       <c r="E11" t="n">
-        <v>0.6482982171799028</v>
+        <v>0.8752025931928687</v>
       </c>
     </row>
   </sheetData>
@@ -1228,7 +1228,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>source: analysis/nh3_mc_ru_actual_2026_10_06/draws.csv (Ru wins: Ru_A_bed &lt; Fe, or Ru_A &lt; Fe); bins of the drawn Ru content</t>
+          <t>source: analysis/nh3_mc_ru_actual_2026_10_06/draws.csv (Ru wins: Ru_A_bed &lt; Fe, or Ru_A &lt; Fe); 5 bins of the drawn A_bed Ru content (A_bed_wt_pct)</t>
         </is>
       </c>
     </row>
@@ -1261,87 +1261,87 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="C4" t="n">
-        <v>283</v>
+        <v>966</v>
       </c>
       <c r="D4" t="n">
-        <v>0</v>
+        <v>0.1966873706004141</v>
       </c>
       <c r="E4" t="n">
-        <v>0.5159010600706714</v>
+        <v>0.6614906832298136</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="B5" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="C5" t="n">
-        <v>1009</v>
+        <v>980</v>
       </c>
       <c r="D5" t="n">
-        <v>0.005946481665014866</v>
+        <v>0.2724489795918367</v>
       </c>
       <c r="E5" t="n">
-        <v>0.5034687809712587</v>
+        <v>0.6520408163265307</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>2.5</v>
+        <v>7</v>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C6" t="n">
-        <v>1967</v>
+        <v>969</v>
       </c>
       <c r="D6" t="n">
-        <v>0.1581087951194713</v>
+        <v>0.3219814241486068</v>
       </c>
       <c r="E6" t="n">
-        <v>0.5292323335027961</v>
+        <v>0.6346749226006192</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C7" t="n">
-        <v>836</v>
+        <v>1012</v>
       </c>
       <c r="D7" t="n">
-        <v>0.3014354066985646</v>
+        <v>0.3527667984189723</v>
       </c>
       <c r="E7" t="n">
-        <v>0.5322966507177034</v>
+        <v>0.6492094861660079</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
+        <v>9</v>
+      </c>
+      <c r="B8" t="n">
         <v>10</v>
       </c>
-      <c r="B8" t="n">
-        <v>15</v>
-      </c>
       <c r="C8" t="n">
-        <v>905</v>
+        <v>1073</v>
       </c>
       <c r="D8" t="n">
-        <v>0.4773480662983425</v>
+        <v>0.3960857409133271</v>
       </c>
       <c r="E8" t="n">
-        <v>0.5093922651933702</v>
+        <v>0.6262814538676608</v>
       </c>
     </row>
   </sheetData>

</xml_diff>